<commit_message>
base de dados excel attualizada
</commit_message>
<xml_diff>
--- a/project/database/TESTE.xlsx
+++ b/project/database/TESTE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cborg\Documents\test\project\database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cborg\test\project\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DF7116-3C62-4974-ADB5-8371054E2193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A26B2A-F665-4B19-A781-88360E4B49E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B81EA3A-3488-412D-A33C-3ACBB3DD87C7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="41">
   <si>
     <t>Nome Produtos</t>
   </si>
@@ -48,13 +48,124 @@
   </si>
   <si>
     <t>segunda</t>
+  </si>
+  <si>
+    <t>Coluna1</t>
+  </si>
+  <si>
+    <t>Coluna2</t>
+  </si>
+  <si>
+    <t>dia 27/07</t>
+  </si>
+  <si>
+    <t>dia 04/08</t>
+  </si>
+  <si>
+    <t>dia 11/08</t>
+  </si>
+  <si>
+    <t>ai</t>
+  </si>
+  <si>
+    <t>ui</t>
+  </si>
+  <si>
+    <t>nmi9dawinja</t>
+  </si>
+  <si>
+    <t>odnjiaw</t>
+  </si>
+  <si>
+    <t>wdawda</t>
+  </si>
+  <si>
+    <t>as</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>terca</t>
+  </si>
+  <si>
+    <t>quarta</t>
+  </si>
+  <si>
+    <t>atg</t>
+  </si>
+  <si>
+    <t>wfg</t>
+  </si>
+  <si>
+    <t>ag</t>
+  </si>
+  <si>
+    <t>ergh</t>
+  </si>
+  <si>
+    <t>rt</t>
+  </si>
+  <si>
+    <t>rj</t>
+  </si>
+  <si>
+    <t>fwq</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>faw</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>tj</t>
+  </si>
+  <si>
+    <t>gw</t>
+  </si>
+  <si>
+    <t>dfwqa</t>
+  </si>
+  <si>
+    <t>hrt</t>
+  </si>
+  <si>
+    <t>her</t>
+  </si>
+  <si>
+    <t>fqw</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>wad</t>
+  </si>
+  <si>
+    <t>quinta</t>
+  </si>
+  <si>
+    <t>sexta</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,6 +184,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -95,16 +212,103 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF9ECE6A"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -118,11 +322,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B0667F17-BF50-4C85-BB0C-E4EEFF7AD150}" name="Tabela1" displayName="Tabela1" ref="A1:B21" totalsRowShown="0">
-  <autoFilter ref="A1:B21" xr:uid="{B0667F17-BF50-4C85-BB0C-E4EEFF7AD150}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{35D4C86D-A418-40D1-9463-08C66C703623}" name="DIA"/>
-    <tableColumn id="2" xr3:uid="{A269FCDB-482A-4CD4-9C5E-49736AA7F922}" name="Nome Produtos"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B0667F17-BF50-4C85-BB0C-E4EEFF7AD150}" name="Tabela1" displayName="Tabela1" ref="A1:G45" totalsRowShown="0">
+  <autoFilter ref="A1:G45" xr:uid="{B0667F17-BF50-4C85-BB0C-E4EEFF7AD150}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{35D4C86D-A418-40D1-9463-08C66C703623}" name="DIA" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{A269FCDB-482A-4CD4-9C5E-49736AA7F922}" name="Nome Produtos" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{A7DEC4FD-1200-4ACE-9FAD-5510315D1A86}" name="dia 27/07" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{9E85EF1F-07E9-4A8E-8439-F0D3737EA417}" name="dia 04/08" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{FC7B458B-98EE-4E25-BC8F-083194B3BB6F}" name="dia 11/08" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{A7BD452F-827A-4440-8266-9F38DCF5F46C}" name="Coluna1" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{EF6B0EC2-8312-4F9B-9D74-BFE764FCDB82}" name="Coluna2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -445,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD2C40FD-A4D7-487E-96E4-4A78EAE8FAD0}">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
@@ -454,173 +663,800 @@
     <col min="10" max="17" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="C2" s="2">
+        <v>123123</v>
+      </c>
+      <c r="D2" s="2">
+        <v>12123</v>
+      </c>
+      <c r="E2" s="2">
+        <v>123123</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3">
+        <v>123</v>
+      </c>
+      <c r="D3" s="3">
+        <v>123</v>
+      </c>
+      <c r="E3" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3">
+        <v>123</v>
+      </c>
+      <c r="D4" s="3">
+        <v>123</v>
+      </c>
+      <c r="E4" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3">
+        <v>123</v>
+      </c>
+      <c r="D5" s="3">
+        <v>123</v>
+      </c>
+      <c r="E5" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3">
+        <v>123</v>
+      </c>
+      <c r="D6" s="3">
+        <v>123</v>
+      </c>
+      <c r="E6" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2">
+        <v>32</v>
+      </c>
+      <c r="C7" s="3">
+        <v>123</v>
+      </c>
+      <c r="D7" s="3">
+        <v>123</v>
+      </c>
+      <c r="E7" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="2">
+        <v>2</v>
+      </c>
+      <c r="C8" s="3">
+        <v>123</v>
+      </c>
+      <c r="D8" s="3">
+        <v>123</v>
+      </c>
+      <c r="E8" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C9" s="3">
+        <v>123</v>
+      </c>
+      <c r="D9" s="3">
+        <v>123</v>
+      </c>
+      <c r="E9" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="C10" s="3">
+        <v>123</v>
+      </c>
+      <c r="D10" s="3">
+        <v>123</v>
+      </c>
+      <c r="E10" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="3">
+        <v>123</v>
+      </c>
+      <c r="D11" s="3">
+        <v>123</v>
+      </c>
+      <c r="E11" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="2">
+        <v>31</v>
+      </c>
+      <c r="C12" s="3">
+        <v>123</v>
+      </c>
+      <c r="D12" s="3">
+        <v>123</v>
+      </c>
+      <c r="E12" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C13" s="3">
+        <v>123</v>
+      </c>
+      <c r="D13" s="3">
+        <v>123</v>
+      </c>
+      <c r="E13" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="3">
+        <v>123</v>
+      </c>
+      <c r="D14" s="3">
+        <v>123</v>
+      </c>
+      <c r="E14" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="3">
+        <v>123</v>
+      </c>
+      <c r="D15" s="3">
+        <v>123</v>
+      </c>
+      <c r="E15" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="C16" s="3">
+        <v>123</v>
+      </c>
+      <c r="D16" s="3">
+        <v>123</v>
+      </c>
+      <c r="E16" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="3">
+        <v>123</v>
+      </c>
+      <c r="D17" s="3">
+        <v>123</v>
+      </c>
+      <c r="E17" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="3">
+        <v>123</v>
+      </c>
+      <c r="D18" s="3">
+        <v>123</v>
+      </c>
+      <c r="E18" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="3">
+        <v>123</v>
+      </c>
+      <c r="D19" s="3">
+        <v>123</v>
+      </c>
+      <c r="E19" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="3">
+        <v>123</v>
+      </c>
+      <c r="D20" s="3">
+        <v>123</v>
+      </c>
+      <c r="E20" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="3">
+        <v>123</v>
+      </c>
+      <c r="D21" s="3">
+        <v>123</v>
+      </c>
+      <c r="E21" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="3">
+        <v>123</v>
+      </c>
+      <c r="D22" s="3">
+        <v>123</v>
+      </c>
+      <c r="E22" s="3">
+        <v>123</v>
+      </c>
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="3">
+        <v>123</v>
+      </c>
+      <c r="D23" s="3">
+        <v>123</v>
+      </c>
+      <c r="E23" s="3">
+        <v>123</v>
+      </c>
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="3">
+        <v>123</v>
+      </c>
+      <c r="D24" s="3">
+        <v>123</v>
+      </c>
+      <c r="E24" s="3">
+        <v>123</v>
+      </c>
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="3">
+        <v>124</v>
+      </c>
+      <c r="D25" s="3">
+        <v>124</v>
+      </c>
+      <c r="E25" s="3">
+        <v>124</v>
+      </c>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="3">
+        <v>51</v>
+      </c>
+      <c r="D26" s="3">
+        <v>51</v>
+      </c>
+      <c r="E26" s="3">
+        <v>51</v>
+      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="3">
+        <v>56</v>
+      </c>
+      <c r="D27" s="3">
+        <v>56</v>
+      </c>
+      <c r="E27" s="3">
+        <v>56</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="3">
+        <v>2356</v>
+      </c>
+      <c r="D28" s="3">
+        <v>2356</v>
+      </c>
+      <c r="E28" s="3">
+        <v>2356</v>
+      </c>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" s="3">
+        <v>24</v>
+      </c>
+      <c r="D29" s="3">
+        <v>24</v>
+      </c>
+      <c r="E29" s="3">
+        <v>24</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="3">
+        <v>124</v>
+      </c>
+      <c r="D30" s="3">
+        <v>124</v>
+      </c>
+      <c r="E30" s="3">
+        <v>124</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="3">
+        <v>14</v>
+      </c>
+      <c r="D31" s="3">
+        <v>14</v>
+      </c>
+      <c r="E31" s="3">
+        <v>14</v>
+      </c>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="3">
+        <v>12</v>
+      </c>
+      <c r="D32" s="3">
+        <v>12</v>
+      </c>
+      <c r="E32" s="3">
+        <v>12</v>
+      </c>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" s="3">
+        <v>143</v>
+      </c>
+      <c r="D33" s="3">
+        <v>143</v>
+      </c>
+      <c r="E33" s="3">
+        <v>143</v>
+      </c>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C34" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="D34" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="E34" s="3">
         <v>1</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="D35" s="3">
         <v>1</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="E35" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="3">
         <v>1</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="D36" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="E36" s="3">
         <v>1</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>1</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>1</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>1</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>1</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>1</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>1</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>1</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>1</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>12</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>1</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>1</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>1</v>
-      </c>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C37" s="3">
+        <v>41</v>
+      </c>
+      <c r="D37" s="3">
+        <v>41</v>
+      </c>
+      <c r="E37" s="3">
+        <v>41</v>
+      </c>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="3">
+        <v>252</v>
+      </c>
+      <c r="D38" s="3">
+        <v>252</v>
+      </c>
+      <c r="E38" s="3">
+        <v>252</v>
+      </c>
+      <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="3">
+        <v>56234</v>
+      </c>
+      <c r="D39" s="3">
+        <v>56234</v>
+      </c>
+      <c r="E39" s="3">
+        <v>56234</v>
+      </c>
+      <c r="F39" s="1"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="3">
+        <v>523</v>
+      </c>
+      <c r="D40" s="3">
+        <v>523</v>
+      </c>
+      <c r="E40" s="3">
+        <v>523</v>
+      </c>
+      <c r="F40" s="1"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C41" s="3">
+        <v>53</v>
+      </c>
+      <c r="D41" s="3">
+        <v>53</v>
+      </c>
+      <c r="E41" s="3">
+        <v>53</v>
+      </c>
+      <c r="F41" s="1"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C42" s="3">
+        <v>6723</v>
+      </c>
+      <c r="D42" s="3">
+        <v>6723</v>
+      </c>
+      <c r="E42" s="3">
+        <v>6723</v>
+      </c>
+      <c r="F42" s="1"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C43" s="3">
+        <v>537</v>
+      </c>
+      <c r="D43" s="3">
+        <v>537</v>
+      </c>
+      <c r="E43" s="3">
+        <v>537</v>
+      </c>
+      <c r="F43" s="1"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C44" s="3">
+        <v>4</v>
+      </c>
+      <c r="D44" s="3">
+        <v>4</v>
+      </c>
+      <c r="E44" s="3">
+        <v>4</v>
+      </c>
+      <c r="F44" s="1"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C45" s="3">
+        <v>63</v>
+      </c>
+      <c r="D45" s="3">
+        <v>63</v>
+      </c>
+      <c r="E45" s="3">
+        <v>63</v>
+      </c>
+      <c r="F45" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>